<commit_message>
5th and ladies final
</commit_message>
<xml_diff>
--- a/Knockouts/5thAndBelow.xlsx
+++ b/Knockouts/5thAndBelow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Ravens Seniors\Knockouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FDAEBF-C885-46B3-B271-8B1876B87A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0828649-8EDE-4777-9673-0B9ECBD98A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1" xr2:uid="{6F46E828-8FFD-4531-838C-1A16471CA10A}"/>
   </bookViews>
@@ -2092,7 +2092,7 @@
         <v>Ravens</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" t="str" cm="1">
         <f t="array" ref="G32:I32">'Knockout Grid'!U36:W36</f>
@@ -2102,7 +2102,7 @@
         <v>CPUT</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>21</v>
@@ -2867,7 +2867,9 @@
       <c r="V35" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="W35" s="11"/>
+      <c r="W35" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
@@ -2886,7 +2888,9 @@
       <c r="V36" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="W36" s="11"/>
+      <c r="W36" s="11">
+        <v>3</v>
+      </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">

</xml_diff>